<commit_message>
fix: remplacer valueCodeableConcept par value.ofType(CodeableConcept) dans les invariants FHIRPath (#489)
* fix: remplacer valueCodeableConcept par value.ofType(CodeableConcept) dans les invariants FHIRPath

Corrige l'erreur "The name 'valueCodeableConcept' is not valid for any of the possible types: [Extension]"
dans les invariants idDecisionMAJCardinality et idDecisionMAJInterdiction.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>

* Fix invariant

---------

Co-authored-by: Claude Sonnet 4.6 <noreply@anthropic.com>
Co-authored-by: TristanKereval <tristan.rieu@kereval.com> 10cd5bba338a7f0d827582f60d5e01febb0e5c05
</commit_message>
<xml_diff>
--- a/main/ig/StructureDefinition-tddui-basic-decision.xlsx
+++ b/main/ig/StructureDefinition-tddui-basic-decision.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-30T14:55:37+00:00</t>
+    <t>2026-07-01T09:47:49+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -267,7 +267,7 @@
   </si>
   <si>
     <t>dom-2:If the resource is contained in another resource, it SHALL NOT contain nested Resources {contained.contained.empty()}
-dom-3:If the resource is contained in another resource, it SHALL be referred to from elsewhere in the resource or SHALL refer to the containing resource {contained.where((('#'+id in (%resource.descendants().reference | %resource.descendants().as(canonical) | %resource.descendants().as(uri) | %resource.descendants().as(url))) or descendants().where(reference = '#').exists() or descendants().where(as(canonical) = '#').exists() or descendants().where(as(canonical) = '#').exists()).not()).trace('unmatched', id).empty()}dom-4:If a resource is contained in another resource, it SHALL NOT have a meta.versionId or a meta.lastUpdated {contained.meta.versionId.empty() and contained.meta.lastUpdated.empty()}dom-5:If a resource is contained in another resource, it SHALL NOT have a security label {contained.meta.security.empty()}dom-6:A resource should have narrative for robust management {text.`div`.exists()}idDecisionMAJCardinality:L'idDecisionMAJ est obligatoire si typeDecision = '5' (Clôture de droit) ou typeDecision ='1' (Attribution) et DroitPrestation.natureDroit = '6' (Renouvellement) ou '7' (Révision). {((extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.where(url='typeDecision').valueCodeableConcept.coding.code='1') and ((extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.where(url='droitPrestation').extension.where(url='natureDroitPrestation').valueCodeableConcept.coding.code='6') or (extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.where(url='droitPrestation').extension.where(url='natureDroitPrestation').valueCodeableConcept.coding.code='7'))) implies (identifier.where(type.coding.code='IDDECISIONMAJ').exists())}idDecisionMAJInterdiction:L'idDecisionMAJ n'est pas à transmettre si typeDecision = '1' (Attribution) et DroitPrestation.natureDroit = '1' (Attribution) {((extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.where(url='typeDecision').valueCodeableConcept.coding.code='1') and (extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.where(url='droitPrestation').extension.where(url='natureDroitPrestation').valueCodeableConcept.coding.code='1')) implies (identifier.where(type.coding.code='IDDECISIONMAJ').exists().not())}</t>
+dom-3:If the resource is contained in another resource, it SHALL be referred to from elsewhere in the resource or SHALL refer to the containing resource {contained.where((('#'+id in (%resource.descendants().reference | %resource.descendants().as(canonical) | %resource.descendants().as(uri) | %resource.descendants().as(url))) or descendants().where(reference = '#').exists() or descendants().where(as(canonical) = '#').exists() or descendants().where(as(canonical) = '#').exists()).not()).trace('unmatched', id).empty()}dom-4:If a resource is contained in another resource, it SHALL NOT have a meta.versionId or a meta.lastUpdated {contained.meta.versionId.empty() and contained.meta.lastUpdated.empty()}dom-5:If a resource is contained in another resource, it SHALL NOT have a security label {contained.meta.security.empty()}dom-6:A resource should have narrative for robust management {text.`div`.exists()}idDecisionMAJCardinality:L'idDecisionMAJ est obligatoire si typeDecision = '5' (Clôture de droit) ou typeDecision ='1' (Attribution) et DroitPrestation.natureDroit = '6' (Renouvellement) ou '7' (Révision). {((extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.where(url='typeDecision').value.ofType(CodeableConcept).coding.code='1') and ((extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.where(url='droitPrestation').extension.where(url='natureDroitPrestation').value.ofType(CodeableConcept).coding.code='6') or (extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.where(url='droitPrestation').extension.where(url='natureDroitPrestation').value.ofType(CodeableConcept).coding.code='7'))) implies (identifier.where(type.coding.code='IDDECISIONMAJ').exists())}idDecisionMAJInterdiction:L'idDecisionMAJ n'est pas à transmettre si typeDecision = '1' (Attribution) et DroitPrestation.natureDroit = '1' (Attribution) {((extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.where(url='typeDecision').value.ofType(CodeableConcept).coding.code='1') and (extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.where(url='droitPrestation').extension.where(url='natureDroitPrestation').value.ofType(CodeableConcept).coding.code='1')) implies (identifier.where(type.coding.code='IDDECISIONMAJ').exists().not())}</t>
   </si>
   <si>
     <t>Decision</t>
@@ -468,7 +468,7 @@
   </si>
   <si>
     <t>ele-1:All FHIR elements must have a @value or children {hasValue() or (children().count() &gt; id.count())}
-ext-1:Must have either extensions or value[x], not both {extension.exists() != value.exists()}motivationLocaleRequired:La motivation locale doit être renseignée si la motivation de la décision est '9999' (Autre). {(extension.where(url='motivation').valueCodeableConcept.coding.where(code='9999').exists()) implies (extension.where(url='motivationLocale').valueString.exists())}DateEffetClotureCardinality:Si typeDecision = '5' (Clôture de droit) alors dateEffetCloture est obligatoire. {(extension.where(url='typeDecision').valueCodeableConcept.coding.where(code='5').exists()) implies (extension.where(url='dateEffetCloture').exists())}</t>
+ext-1:Must have either extensions or value[x], not both {extension.exists() != value.exists()}motivationLocaleRequired:La motivation locale doit être renseignée si la motivation de la décision est '9999' (Autre). {(extension.where(url='motivation').value.ofType(CodeableConcept).coding.where(code='9999').exists()) implies (extension.where(url='motivationLocale').value.ofType(String).exists())}DateEffetClotureCardinality:Si typeDecision = '5' (Clôture de droit) alors dateEffetCloture est obligatoire. {(extension.where(url='typeDecision').value.ofType(CodeableConcept).coding.where(code='5').exists()) implies (extension.where(url='dateEffetCloture').exists())}</t>
   </si>
   <si>
     <t>Basic.extension:TDDUIDecision.id</t>
@@ -688,8 +688,8 @@
   </si>
   <si>
     <t>ele-1:All FHIR elements must have a @value or children {hasValue() or (children().count() &gt; id.count())}
-ext-1:Must have either extensions or value[x], not both {extension.exists() != value.exists()}FormationCardinality:Formation est obligatoire si typeDroitPrestation = '11.1' (Orientation en Centre de rééducation professionnelle (CRP)). {(extension.where(url='typeDroitPrestation').valueCodeableConcept.coding.code='11.1') implies (extension.where(url='droitPrestation').extension.where(url='detailPrestation').extension.where(url='formation'))}PrecisionOrientationValues7.8:Si typeDroitPrestation = '7.8' (Orientation vers un Service d'éducation spéciale et de soins à domicile (SESSAD)) alors precisionOrientation entre '1' et
- '6' {(extension.where(url='typeDroitPrestation').valueCodeableConcept.coding.code='7.8') implies ((extension.where(url='detailPrestation').extension.where(url='precisionOrientation').valueCodeableConcept.coding.code.toInteger()&gt;=1) and (extension.where(url='detailPrestation').extension.where(url='precisionOrientation').valueCodeableConcept.coding.code.toInteger()&lt;=6))}PrecisionOrientationValues7.9:Si typeDroitPrestation = '7.9' (Orientation vers un Service d'accompagnement familial et d'éducation précoce (SAFEP)) alors precisionOrientation entre '7' et '8' {(extension.where(url='typeDroitPrestation').valueCodeableConcept.coding.code='7.9') implies ((extension.where(url='detailPrestation').extension.where(url='precisionOrientation').valueCodeableConcept.coding.code.toInteger()&gt;=7) and (extension.where(url='detailPrestation').extension.where(url='precisionOrientation').valueCodeableConcept.coding.code.toInteger()&lt;=8))}PrecisionOrientationValues13.1-13.2:Si typeDroitPrestation = '13.1' (Orientation vers un établissement d'accueil non médicalisé) ou '13.2' (Orientation vers un établissement d'accueil médicalisé en tout ou partie) alors precisionOrientation est interdit {((extension.where(url='typeDroitPrestation').valueCodeableConcept.coding.code='13.1') or (extension.where(url='typeDroitPrestation').valueCodeableConcept.coding.code='13.2')) implies (extension.where(url='detailPrestation').extension.where(url='precisionOrientation').not())}PrecisionOrientationValues8.3:Si typeDroitPrestation = '8.3' (Orientation en Enseignement adapté (SEGPA/EREA)) alors precisionOrientation entre '9' et '10'  {(extension.where(url='typeDroitPrestation').valueCodeableConcept.coding.code='8.3') implies ((extension.where(url='detailPrestation').extension.where(url='precisionOrientation').valueCodeableConcept.coding.code.toInteger()&gt;=9) and (extension.where(url='detailPrestation').extension.where(url='precisionOrientation').valueCodeableConcept.coding.code.toInteger()&lt;=10))}PrecisionOrientationValues8.6:Si typeDroitPrestation = '8.6' (Orientation en Unité d'enseignement) alors precisionOrientation = 'UEA' (Unité d'enseignement élémentaire autisme) ou 'UEM' (Unité d'enseignement en maternelle plan autisme). {(extension.where(url='typeDroitPrestation').valueCodeableConcept.coding.code='8.6') implies ((extension.where(url='detailPrestation').extension.where(url='precisionOrientation').valueCodeableConcept.coding.code='UEA') or (extension.where(url='detailPrestation').extension.where(url='precisionOrientation').valueCodeableConcept.coding.code='UEM'))}temporaliteAccueilCardinalityViaCategorieDroitPrestation:Si categorieDroitPrestation = '13' (Orientation ESMS Adultes) ou '7' (Orientation ESMS Enfants) alors temporaliteAccueil est obligatoire. {((extension.where(url='categorieDroitPrestation').valueCodeableConcept.coding.code='13') or (extension.where(url='categorieDroitPrestation').valueCodeableConcept.coding.code='7')) implies (extension.where(url='detailPrestation').extension.where(url='temporaliteAccueil'))}temporaliteAccueilCardinalityViaTypeDroitPrestation:Si typeDroitPrestation = '8.6' (Orientation en Unité d'enseignement) ou '8.7' (Orientation vers une Scolarisation en milieu ordinaire à temps partagé) ou '8.8' (Orientation vers une Unité d'enseignement et une scolarisation en ULIS à temps partagé) ou '8.10' (Orientation vers une unité d'enseignement et une scolarisation en enseignement adapté à temps partagé) alors la temporalité d'accueil est obligatoire. {((extension.where(url='typeDroitPrestation').valueCodeableConcept.coding.code='8.6') or (extension.where(url='typeDroitPrestation').valueCodeableConcept.coding.code='8.7') or (extension.where(url='typeDroitPrestation').valueCodeableConcept.coding.code='8.8') or (extension.where(url='typeDroitPrestation').valueCodeableConcept.coding.code='8.10')) implies (extension.where(url='droitPrestation').extension.where(url='detailPrestation').extension.where(url='temporaliteAccueil'))}cretonCardinality:Si categorieDroitPrestation = '7' (ESSMS enfant) alors Creton est obligatoire {((extension.where(url='categorieDroitPrestation').valueCodeableConcept.coding.code='7') or (extension.where(url='typeDroitPrestation').valueCodeableConcept.coding.code.matches('^7[.][0-9]+$'))) implies (extension.where(url='creton'))}</t>
+ext-1:Must have either extensions or value[x], not both {extension.exists() != value.exists()}FormationCardinality:Formation est obligatoire si typeDroitPrestation = '11.1' (Orientation en Centre de rééducation professionnelle (CRP)). {(extension.where(url='typeDroitPrestation').value.ofType(CodeableConcept).coding.code='11.1') implies (extension.where(url='droitPrestation').extension.where(url='detailPrestation').extension.where(url='formation'))}PrecisionOrientationValues7.8:Si typeDroitPrestation = '7.8' (Orientation vers un Service d'éducation spéciale et de soins à domicile (SESSAD)) alors precisionOrientation entre '1' et
+ '6' {(extension.where(url='typeDroitPrestation').value.ofType(CodeableConcept).coding.code='7.8') implies ((extension.where(url='detailPrestation').extension.where(url='precisionOrientation').value.ofType(CodeableConcept).coding.code.toInteger()&gt;=1) and (extension.where(url='detailPrestation').extension.where(url='precisionOrientation').value.ofType(CodeableConcept).coding.code.toInteger()&lt;=6))}PrecisionOrientationValues7.9:Si typeDroitPrestation = '7.9' (Orientation vers un Service d'accompagnement familial et d'éducation précoce (SAFEP)) alors precisionOrientation entre '7' et '8' {(extension.where(url='typeDroitPrestation').value.ofType(CodeableConcept).coding.code='7.9') implies ((extension.where(url='detailPrestation').extension.where(url='precisionOrientation').value.ofType(CodeableConcept).coding.code.toInteger()&gt;=7) and (extension.where(url='detailPrestation').extension.where(url='precisionOrientation').value.ofType(CodeableConcept).coding.code.toInteger()&lt;=8))}PrecisionOrientationValues13.1-13.2:Si typeDroitPrestation = '13.1' (Orientation vers un établissement d'accueil non médicalisé) ou '13.2' (Orientation vers un établissement d'accueil médicalisé en tout ou partie) alors precisionOrientation est interdit {((extension.where(url='typeDroitPrestation').value.ofType(CodeableConcept).coding.code='13.1') or (extension.where(url='typeDroitPrestation').value.ofType(CodeableConcept).coding.code='13.2')) implies (extension.where(url='detailPrestation').extension.where(url='precisionOrientation').not())}PrecisionOrientationValues8.3:Si typeDroitPrestation = '8.3' (Orientation en Enseignement adapté (SEGPA/EREA)) alors precisionOrientation entre '9' et '10'  {(extension.where(url='typeDroitPrestation').value.ofType(CodeableConcept).coding.code='8.3') implies ((extension.where(url='detailPrestation').extension.where(url='precisionOrientation').value.ofType(CodeableConcept).coding.code.toInteger()&gt;=9) and (extension.where(url='detailPrestation').extension.where(url='precisionOrientation').value.ofType(CodeableConcept).coding.code.toInteger()&lt;=10))}PrecisionOrientationValues8.6:Si typeDroitPrestation = '8.6' (Orientation en Unité d'enseignement) alors precisionOrientation = 'UEA' (Unité d'enseignement élémentaire autisme) ou 'UEM' (Unité d'enseignement en maternelle plan autisme). {(extension.where(url='typeDroitPrestation').value.ofType(CodeableConcept).coding.code='8.6') implies ((extension.where(url='detailPrestation').extension.where(url='precisionOrientation').value.ofType(CodeableConcept).coding.code='UEA') or (extension.where(url='detailPrestation').extension.where(url='precisionOrientation').value.ofType(CodeableConcept).coding.code='UEM'))}temporaliteAccueilCardinalityViaCategorieDroitPrestation:Si categorieDroitPrestation = '13' (Orientation ESMS Adultes) ou '7' (Orientation ESMS Enfants) alors temporaliteAccueil est obligatoire. {((extension.where(url='categorieDroitPrestation').value.ofType(CodeableConcept).coding.code='13') or (extension.where(url='categorieDroitPrestation').value.ofType(CodeableConcept).coding.code='7')) implies (extension.where(url='detailPrestation').extension.where(url='temporaliteAccueil'))}temporaliteAccueilCardinalityViaTypeDroitPrestation:Si typeDroitPrestation = '8.6' (Orientation en Unité d'enseignement) ou '8.7' (Orientation vers une Scolarisation en milieu ordinaire à temps partagé) ou '8.8' (Orientation vers une Unité d'enseignement et une scolarisation en ULIS à temps partagé) ou '8.10' (Orientation vers une unité d'enseignement et une scolarisation en enseignement adapté à temps partagé) alors la temporalité d'accueil est obligatoire. {((extension.where(url='typeDroitPrestation').value.ofType(CodeableConcept).coding.code='8.6') or (extension.where(url='typeDroitPrestation').value.ofType(CodeableConcept).coding.code='8.7') or (extension.where(url='typeDroitPrestation').value.ofType(CodeableConcept).coding.code='8.8') or (extension.where(url='typeDroitPrestation').value.ofType(CodeableConcept).coding.code='8.10')) implies (extension.where(url='droitPrestation').extension.where(url='detailPrestation').extension.where(url='temporaliteAccueil'))}cretonCardinality:Si categorieDroitPrestation = '7' (ESSMS enfant) alors Creton est obligatoire {((extension.where(url='categorieDroitPrestation').value.ofType(CodeableConcept).coding.code='7') or (extension.where(url='typeDroitPrestation').value.ofType(CodeableConcept).coding.code.matches('^7[.][0-9]+$'))) implies (extension.where(url='creton'))}</t>
   </si>
   <si>
     <t>DroitPrestation</t>

</xml_diff>

<commit_message>
Fix fhirpath value codeable concept (#490)
* fix: remplacer valueCodeableConcept par value.ofType(CodeableConcept) dans les invariants FHIRPath

Corrige l'erreur "The name 'valueCodeableConcept' is not valid for any of the possible types: [Extension]"
dans les invariants idDecisionMAJCardinality et idDecisionMAJInterdiction.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>

* Fix invariant

* Fix QA

---------

Co-authored-by: Nicolas Riss <48218773+nriss@users.noreply.github.com>
Co-authored-by: Claude Sonnet 4.6 <noreply@anthropic.com> 611f006ddcadc6774e33a39e9b29aed79e2d8dc8
</commit_message>
<xml_diff>
--- a/main/ig/StructureDefinition-tddui-basic-decision.xlsx
+++ b/main/ig/StructureDefinition-tddui-basic-decision.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-07-01T09:47:49+00:00</t>
+    <t>2026-07-01T11:47:31+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -468,7 +468,7 @@
   </si>
   <si>
     <t>ele-1:All FHIR elements must have a @value or children {hasValue() or (children().count() &gt; id.count())}
-ext-1:Must have either extensions or value[x], not both {extension.exists() != value.exists()}motivationLocaleRequired:La motivation locale doit être renseignée si la motivation de la décision est '9999' (Autre). {(extension.where(url='motivation').value.ofType(CodeableConcept).coding.where(code='9999').exists()) implies (extension.where(url='motivationLocale').value.ofType(String).exists())}DateEffetClotureCardinality:Si typeDecision = '5' (Clôture de droit) alors dateEffetCloture est obligatoire. {(extension.where(url='typeDecision').value.ofType(CodeableConcept).coding.where(code='5').exists()) implies (extension.where(url='dateEffetCloture').exists())}</t>
+ext-1:Must have either extensions or value[x], not both {extension.exists() != value.exists()}motivationLocaleRequired:La motivation locale doit être renseignée si la motivation de la décision est '9999' (Autre). {(extension.where(url='motivation').value.ofType(CodeableConcept).coding.where(code='9999').exists()) implies (extension.where(url='motivationLocale').value.ofType(string).exists())}DateEffetClotureCardinality:Si typeDecision = '5' (Clôture de droit) alors dateEffetCloture est obligatoire. {(extension.where(url='typeDecision').value.ofType(CodeableConcept).coding.where(code='5').exists()) implies (extension.where(url='dateEffetCloture').exists())}</t>
   </si>
   <si>
     <t>Basic.extension:TDDUIDecision.id</t>

</xml_diff>

<commit_message>
ANS-009-004 Fix invariant (#494)
* Fix invariant

* Fix invariant

* Fix invariant

* Fix invariant 5e122f5bf0fa1f9e2f5d642c060ebd1c27d264d5
</commit_message>
<xml_diff>
--- a/main/ig/StructureDefinition-tddui-basic-decision.xlsx
+++ b/main/ig/StructureDefinition-tddui-basic-decision.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-07-01T15:33:30+00:00</t>
+    <t>2026-07-20T07:42:46+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -267,7 +267,47 @@
   </si>
   <si>
     <t>dom-2:If the resource is contained in another resource, it SHALL NOT contain nested Resources {contained.contained.empty()}
-dom-3:If the resource is contained in another resource, it SHALL be referred to from elsewhere in the resource or SHALL refer to the containing resource {contained.where((('#'+id in (%resource.descendants().reference | %resource.descendants().as(canonical) | %resource.descendants().as(uri) | %resource.descendants().as(url))) or descendants().where(reference = '#').exists() or descendants().where(as(canonical) = '#').exists() or descendants().where(as(canonical) = '#').exists()).not()).trace('unmatched', id).empty()}dom-4:If a resource is contained in another resource, it SHALL NOT have a meta.versionId or a meta.lastUpdated {contained.meta.versionId.empty() and contained.meta.lastUpdated.empty()}dom-5:If a resource is contained in another resource, it SHALL NOT have a security label {contained.meta.security.empty()}dom-6:A resource should have narrative for robust management {text.`div`.exists()}idDecisionMAJCardinality:L'idDecisionMAJ est obligatoire si typeDecision = '5' (Clôture de droit) ou typeDecision ='1' (Attribution) et DroitPrestation.natureDroit = '6' (Renouvellement) ou '7' (Révision). {((extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.where(url='typeDecision').value.ofType(CodeableConcept).coding.code='1') and ((extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.where(url='droitPrestation').extension.where(url='natureDroitPrestation').value.ofType(CodeableConcept).coding.code='6') or (extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.where(url='droitPrestation').extension.where(url='natureDroitPrestation').value.ofType(CodeableConcept).coding.code='7'))) implies (identifier.where(type.coding.code='IDDECISIONMAJ').exists())}idDecisionMAJInterdiction:L'idDecisionMAJ n'est pas à transmettre si typeDecision = '1' (Attribution) et DroitPrestation.natureDroit = '1' (Attribution) {((extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.where(url='typeDecision').value.ofType(CodeableConcept).coding.code='1') and (extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.where(url='droitPrestation').extension.where(url='natureDroitPrestation').value.ofType(CodeableConcept).coding.code='1')) implies (identifier.where(type.coding.code='IDDECISIONMAJ').exists().not())}</t>
+dom-3:If the resource is contained in another resource, it SHALL be referred to from elsewhere in the resource or SHALL refer to the containing resource {contained.where((('#'+id in (%resource.descendants().reference | %resource.descendants().as(canonical) | %resource.descendants().as(uri) | %resource.descendants().as(url))) or descendants().where(reference = '#').exists() or descendants().where(as(canonical) = '#').exists() or descendants().where(as(canonical) = '#').exists()).not()).trace('unmatched', id).empty()}dom-4:If a resource is contained in another resource, it SHALL NOT have a meta.versionId or a meta.lastUpdated {contained.meta.versionId.empty() and contained.meta.lastUpdated.empty()}dom-5:If a resource is contained in another resource, it SHALL NOT have a security label {contained.meta.security.empty()}dom-6:A resource should have narrative for robust management {text.`div`.exists()}idDecisionMAJCardinality:L'idDecisionMAJ est obligatoire si typeDecision = '5' (Clôture de droit) ou typeDecision ='1' (Attribution) et DroitPrestation.natureDroit = '6' (Renouvellement) ou '7' (Révision). {(
+  iif(
+    extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').exists(),
+    (
+      extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.where(url='typeDecision').value.ofType(CodeableConcept).coding.where(code='5').exists()
+      or
+      (
+        extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.where(url='typeDecision').value.ofType(CodeableConcept).coding.where(code='1').exists()
+        and
+        iif(
+          extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.where(url='droitPrestation').exists(),
+          (
+            extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.where(url='droitPrestation').extension.where(url='natureDroitPrestation').value.ofType(CodeableConcept).coding.where(code='6').exists()
+            or
+            extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.where(url='droitPrestation').extension.where(url='natureDroitPrestation').value.ofType(CodeableConcept).coding.where(code='7').exists()
+          ),
+          false
+        )
+      )
+    ),
+    false
+  )
+)
+implies
+(
+  identifier.where(type.coding.code='IDDECISIONMAJ').exists()
+)}idDecisionMAJInterdiction:L'idDecisionMAJ n'est pas à transmettre si typeDecision = '1' (Attribution) et DroitPrestation.natureDroit = '1' (Attribution) {(
+  iif(
+    extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').exists(),
+    (
+      extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.where(url='typeDecision').value.ofType(CodeableConcept).coding.where(code='1').exists()
+      and
+      extension.where(url='https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-decision').extension.where(url='droitPrestation').extension.where(url='natureDroitPrestation').value.ofType(CodeableConcept).coding.where(code='1').exists()
+    ),
+    false
+  )
+)
+implies
+(
+  identifier.where(type.coding.code='IDDECISIONMAJ').exists().not()
+)}</t>
   </si>
   <si>
     <t>Decision</t>
@@ -688,8 +728,40 @@
   </si>
   <si>
     <t>ele-1:All FHIR elements must have a @value or children {hasValue() or (children().count() &gt; id.count())}
-ext-1:Must have either extensions or value[x], not both {extension.exists() != value.exists()}FormationCardinality:Formation est obligatoire si typeDroitPrestation = '11.1' (Orientation en Centre de rééducation professionnelle (CRP)). {(extension.where(url='typeDroitPrestation').value.ofType(CodeableConcept).coding.code='11.1') implies (extension.where(url='droitPrestation').extension.where(url='detailPrestation').extension.where(url='formation'))}PrecisionOrientationValues7.8:Si typeDroitPrestation = '7.8' (Orientation vers un Service d'éducation spéciale et de soins à domicile (SESSAD)) alors precisionOrientation entre '1' et
- '6' {(extension.where(url='typeDroitPrestation').value.ofType(CodeableConcept).coding.code='7.8') implies ((extension.where(url='detailPrestation').extension.where(url='precisionOrientation').value.ofType(CodeableConcept).coding.code.toInteger()&gt;=1) and (extension.where(url='detailPrestation').extension.where(url='precisionOrientation').value.ofType(CodeableConcept).coding.code.toInteger()&lt;=6))}PrecisionOrientationValues7.9:Si typeDroitPrestation = '7.9' (Orientation vers un Service d'accompagnement familial et d'éducation précoce (SAFEP)) alors precisionOrientation entre '7' et '8' {(extension.where(url='typeDroitPrestation').value.ofType(CodeableConcept).coding.code='7.9') implies ((extension.where(url='detailPrestation').extension.where(url='precisionOrientation').value.ofType(CodeableConcept).coding.code.toInteger()&gt;=7) and (extension.where(url='detailPrestation').extension.where(url='precisionOrientation').value.ofType(CodeableConcept).coding.code.toInteger()&lt;=8))}PrecisionOrientationValues13.1-13.2:Si typeDroitPrestation = '13.1' (Orientation vers un établissement d'accueil non médicalisé) ou '13.2' (Orientation vers un établissement d'accueil médicalisé en tout ou partie) alors precisionOrientation est interdit {((extension.where(url='typeDroitPrestation').value.ofType(CodeableConcept).coding.code='13.1') or (extension.where(url='typeDroitPrestation').value.ofType(CodeableConcept).coding.code='13.2')) implies (extension.where(url='detailPrestation').extension.where(url='precisionOrientation').not())}PrecisionOrientationValues8.3:Si typeDroitPrestation = '8.3' (Orientation en Enseignement adapté (SEGPA/EREA)) alors precisionOrientation entre '9' et '10'  {(extension.where(url='typeDroitPrestation').value.ofType(CodeableConcept).coding.code='8.3') implies ((extension.where(url='detailPrestation').extension.where(url='precisionOrientation').value.ofType(CodeableConcept).coding.code.toInteger()&gt;=9) and (extension.where(url='detailPrestation').extension.where(url='precisionOrientation').value.ofType(CodeableConcept).coding.code.toInteger()&lt;=10))}PrecisionOrientationValues8.6:Si typeDroitPrestation = '8.6' (Orientation en Unité d'enseignement) alors precisionOrientation = 'UEA' (Unité d'enseignement élémentaire autisme) ou 'UEM' (Unité d'enseignement en maternelle plan autisme). {(extension.where(url='typeDroitPrestation').value.ofType(CodeableConcept).coding.code='8.6') implies ((extension.where(url='detailPrestation').extension.where(url='precisionOrientation').value.ofType(CodeableConcept).coding.code='UEA') or (extension.where(url='detailPrestation').extension.where(url='precisionOrientation').value.ofType(CodeableConcept).coding.code='UEM'))}temporaliteAccueilCardinalityViaCategorieDroitPrestation:Si categorieDroitPrestation = '13' (Orientation ESMS Adultes) ou '7' (Orientation ESMS Enfants) alors temporaliteAccueil est obligatoire. {((extension.where(url='categorieDroitPrestation').value.ofType(CodeableConcept).coding.code='13') or (extension.where(url='categorieDroitPrestation').value.ofType(CodeableConcept).coding.code='7')) implies (extension.where(url='detailPrestation').extension.where(url='temporaliteAccueil'))}temporaliteAccueilCardinalityViaTypeDroitPrestation:Si typeDroitPrestation = '8.6' (Orientation en Unité d'enseignement) ou '8.7' (Orientation vers une Scolarisation en milieu ordinaire à temps partagé) ou '8.8' (Orientation vers une Unité d'enseignement et une scolarisation en ULIS à temps partagé) ou '8.10' (Orientation vers une unité d'enseignement et une scolarisation en enseignement adapté à temps partagé) alors la temporalité d'accueil est obligatoire. {((extension.where(url='typeDroitPrestation').value.ofType(CodeableConcept).coding.code='8.6') or (extension.where(url='typeDroitPrestation').value.ofType(CodeableConcept).coding.code='8.7') or (extension.where(url='typeDroitPrestation').value.ofType(CodeableConcept).coding.code='8.8') or (extension.where(url='typeDroitPrestation').value.ofType(CodeableConcept).coding.code='8.10')) implies (extension.where(url='droitPrestation').extension.where(url='detailPrestation').extension.where(url='temporaliteAccueil'))}cretonCardinality:Si categorieDroitPrestation = '7' (ESSMS enfant) alors Creton est obligatoire {((extension.where(url='categorieDroitPrestation').value.ofType(CodeableConcept).coding.code='7') or (extension.where(url='typeDroitPrestation').value.ofType(CodeableConcept).coding.code.matches('^7[.][0-9]+$'))) implies (extension.where(url='creton'))}</t>
+ext-1:Must have either extensions or value[x], not both {extension.exists() != value.exists()}FormationCardinality:Formation est obligatoire si typeDroitPrestation = '11.1' (Orientation en Centre de rééducation professionnelle (CRP)). {(extension.where(url='typeDroitPrestation').value.ofType(CodeableConcept).coding.where(code='11.1').exists()) implies (extension.where(url='droitPrestation').extension.where(url='detailPrestation').extension.where(url='formation').exists())}PrecisionOrientationValues7.8:Si typeDroitPrestation = '7.8' (Orientation vers un Service d'éducation spéciale et de soins à domicile (SESSAD)) alors precisionOrientation doit être entre '1' et
+ '6' {(
+  extension.where(url='typeDroitPrestation').value.ofType(CodeableConcept).coding.where(code='7.8').exists()
+  and
+  extension.where(url='detailPrestation').extension.where(url='precisionOrientation').exists()
+)
+implies
+(
+  extension.where(url='detailPrestation').extension.where(url='precisionOrientation').value.ofType(CodeableConcept).coding.where(code='1' or code='2' or code='3' or code='4' or code='5' or code='6').exists()
+)}PrecisionOrientationValues7.9:Si typeDroitPrestation = '7.9' (Orientation vers un Service d'accompagnement familial et d'éducation précoce (SAFEP)) alors precisionOrientation doit être entre '7' et '8' {(
+  extension.where(url='typeDroitPrestation').value.ofType(CodeableConcept).coding.where(code='7.9').exists()
+  and
+  extension.where(url='detailPrestation').extension.where(url='precisionOrientation').exists()
+)
+implies
+(
+  extension.where(url='detailPrestation').extension.where(url='precisionOrientation').value.ofType(CodeableConcept).coding.where(code='7' or code='8').exists()
+)}PrecisionOrientationValues13.1-13.2:Si typeDroitPrestation = '13.1' (Orientation vers un établissement d'accueil non médicalisé) ou '13.2' (Orientation vers un établissement d'accueil médicalisé en tout ou partie) alors precisionOrientation est interdit {((extension.where(url='typeDroitPrestation').value.ofType(CodeableConcept).coding.where(code='13.1').exists()) or (extension.where(url='typeDroitPrestation').value.ofType(CodeableConcept).coding.where(code='13.2').exists())) implies (extension.where(url='detailPrestation').extension.where(url='precisionOrientation').exists().not())}PrecisionOrientationValues8.3:Si typeDroitPrestation = '8.3' (Orientation en Enseignement adapté (SEGPA/EREA)) alors precisionOrientation doit être entre '9' et '10'  {(
+  extension.where(url='typeDroitPrestation').value.ofType(CodeableConcept).coding.where(code='8.3').exists()
+  and
+  extension.where(url='detailPrestation').extension.where(url='precisionOrientation').exists()
+)
+implies
+(
+  extension.where(url='detailPrestation').extension.where(url='precisionOrientation').value.ofType(CodeableConcept).coding.where(code='9' or code='10').exists()
+)}PrecisionOrientationValues8.6:Si typeDroitPrestation = '8.6' (Orientation en Unité d'enseignement) alors precisionOrientation = 'UEA' (Unité d'enseignement élémentaire autisme) ou 'UEM' (Unité d'enseignement en maternelle plan autisme). {(
+  extension.where(url='typeDroitPrestation').value.ofType(CodeableConcept).coding.where(code='8.6').exists()
+  and
+  extension.where(url='detailPrestation').extension.where(url='precisionOrientation').exists()
+)
+implies
+(
+  extension.where(url='detailPrestation').extension.where(url='precisionOrientation').value.ofType(CodeableConcept).coding.where(code='UEA' or code='UEM').exists()
+)}temporaliteAccueilCardinalityViaCategorieDroitPrestation:Si categorieDroitPrestation = '13' (Orientation ESMS Adultes) ou '7' (Orientation ESMS Enfants) alors temporaliteAccueil est obligatoire. {((extension.where(url='categorieDroitPrestation').value.ofType(CodeableConcept).coding.where(code='13').exists()) or (extension.where(url='categorieDroitPrestation').value.ofType(CodeableConcept).coding.where(code='7')).exists()) implies (extension.where(url='detailPrestation').extension.where(url='temporaliteAccueil').exists())}temporaliteAccueilCardinalityViaTypeDroitPrestation:Si typeDroitPrestation = '8.6' (Orientation en Unité d'enseignement) ou '8.7' (Orientation vers une Scolarisation en milieu ordinaire à temps partagé) ou '8.8' (Orientation vers une Unité d'enseignement et une scolarisation en ULIS à temps partagé) ou '8.10' (Orientation vers une unité d'enseignement et une scolarisation en enseignement adapté à temps partagé) alors la temporalité d'accueil est obligatoire. {((extension.where(url='typeDroitPrestation').value.ofType(CodeableConcept).coding.where(code='8.6').exists()) or (extension.where(url='typeDroitPrestation').value.ofType(CodeableConcept).coding.where(code='8.7').exists()) or (extension.where(url='typeDroitPrestation').value.ofType(CodeableConcept).coding.where(code='8.8').exists()) or (extension.where(url='typeDroitPrestation').value.ofType(CodeableConcept).coding.where(code='8.10').exists())) implies (extension.where(url='droitPrestation').extension.where(url='detailPrestation').extension.where(url='temporaliteAccueil').exists())}cretonCardinality:Si categorieDroitPrestation = '7' (ESSMS enfant) alors Creton est obligatoire {((extension.where(url='categorieDroitPrestation').value.ofType(CodeableConcept).coding.where(code='7').exists()) or (extension.where(url='typeDroitPrestation').value.ofType(CodeableConcept).coding.code.matches('^7[.][0-9]+$'))) implies (extension.where(url='creton').exists())}</t>
   </si>
   <si>
     <t>DroitPrestation</t>

</xml_diff>